<commit_message>
feat: add employee email mapping and dynamic avatar photo integration
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3501,7 +3501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3525,6 +3525,11 @@
           <t>Role</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -3547,6 +3552,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Lam.Le@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -3569,6 +3579,11 @@
           <t>Super User</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>khuong.ngo@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -3591,6 +3606,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Wynn.Nguyen@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -3613,6 +3633,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Wendy.Nguyen@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -3635,6 +3660,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Hannah.Dinh@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -3657,6 +3687,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Austin.Nguyen@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -3679,6 +3714,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mia.Tran@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -3701,6 +3741,11 @@
           <t>Employee</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Trung.Nguyen@AreteEPM.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -3721,6 +3766,11 @@
       <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Manager</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Hanoi.Office@AreteEPM.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add authentication, login shield, password change, and SMTP password reset
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -328,7 +328,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="51.5" customWidth="1" style="3" min="2" max="2"/>
@@ -405,7 +405,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="2">
-        <f>IF(G2, TEXT(F2/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G2, TEXT(F2/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -437,39 +437,40 @@
         <v>1</v>
       </c>
       <c r="H3" s="2">
-        <f>IF(G3, TEXT(F3/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G3, TEXT(F3/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>What's New in Financial Consolidation and Close</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>25m</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2">
-        <f>IF(G4, TEXT(F4/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="C4" s="0" t="inlineStr"/>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Oracle SmartView For Financial Consolidation and Close</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>2h 40m</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>160</v>
+      </c>
+      <c r="G4" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="0">
+        <f>IF(G4, TEXT(F4/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -486,22 +487,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>What's New in Financial Consolidation and Close</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>158</v>
+        <v>25</v>
       </c>
       <c r="G5" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H5" s="2">
-        <f>IF(G5, TEXT(F5/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G5, TEXT(F5/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -518,22 +519,22 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1h 31m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>91</v>
+        <v>158</v>
       </c>
       <c r="G6" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H6" s="2">
-        <f>IF(G6, TEXT(F6/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G6, TEXT(F6/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -545,59 +546,60 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified PCM Implementer</t>
+          <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM: Enterprise Profitability and Cost Management</t>
+          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>14h 20m</t>
+          <t>1h 31m</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>860</v>
+        <v>91</v>
       </c>
       <c r="G7" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H7" s="2">
-        <f>IF(G7, TEXT(F7/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G7, TEXT(F7/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Become a Certified PCM Implementer</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>What's New in Enterprise Profitability and Cost Management</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>47m</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="G8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2">
-        <f>IF(G8, TEXT(F8/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr"/>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>1h 30m</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="0">
+        <f>IF(G8, TEXT(F8/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -614,22 +616,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Oracle Cloud EPM: Enterprise Profitability and Cost Management</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>14h 20m</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>158</v>
+        <v>860</v>
       </c>
       <c r="G9" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H9" s="2">
-        <f>IF(G9, TEXT(F9/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G9, TEXT(F9/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -646,22 +648,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Oracle Profitability and Cost Management 2026 Implementation Professional (1Z0-1082-26)</t>
+          <t>What's New in Enterprise Profitability and Cost Management</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>47m</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="G10" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H10" s="2">
-        <f>IF(G10, TEXT(F10/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G10, TEXT(F10/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -673,27 +675,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Narrative Reporting Implementer</t>
+          <t>Become a Certified PCM Implementer</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Creating Reports in Cloud EPM</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2h 21m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="G11" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H11" s="2">
-        <f>IF(G11, TEXT(F11/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G11, TEXT(F11/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -705,27 +707,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Narrative Reporting Implementer</t>
+          <t>Become a Certified PCM Implementer</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Narrative Reporting Overview and Administration</t>
+          <t>Oracle Profitability and Cost Management 2026 Implementation Professional (1Z0-1082-26)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>1h 39m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G12" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H12" s="2">
-        <f>IF(G12, TEXT(F12/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G12, TEXT(F12/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -742,22 +744,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Create and Manage Report Packages in Narrative Reporting</t>
+          <t>Creating Reports in Cloud EPM</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2h 0m</t>
+          <t>2h 21m</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="G13" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H13" s="2">
-        <f>IF(G13, TEXT(F13/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G13, TEXT(F13/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -774,22 +776,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>What's New in Narrative Reporting</t>
+          <t>Narrative Reporting Overview and Administration</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>35m</t>
+          <t>1h 39m</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="G14" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H14" s="2">
-        <f>IF(G14, TEXT(F14/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G14, TEXT(F14/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -806,22 +808,22 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Create and Manage Report Packages in Narrative Reporting</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>2h 0m</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="G15" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H15" s="2">
-        <f>IF(G15, TEXT(F15/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G15, TEXT(F15/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -838,22 +840,22 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Oracle Narrative Reporting 2025 Implementation Professional (1Z0-1083-25-JPN)</t>
+          <t>What's New in Narrative Reporting</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>1h 31m</t>
+          <t>35m</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="G16" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H16" s="2">
-        <f>IF(G16, TEXT(F16/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G16, TEXT(F16/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -870,22 +872,22 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Oracle Narrative Reporting 2026 Implementation Professional (1Z0-1083-26)</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>90</v>
+        <v>158</v>
       </c>
       <c r="G17" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H17" s="2">
-        <f>IF(G17, TEXT(F17/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G17, TEXT(F17/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -897,27 +899,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified Narrative Reporting Implementer</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Integrating Data in Cloud EPM</t>
+          <t>Oracle Narrative Reporting 2025 Implementation Professional (1Z0-1083-25-JPN)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4h 43m</t>
+          <t>1h 31m</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>283</v>
+        <v>91</v>
       </c>
       <c r="G18" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H18" s="2">
-        <f>IF(G18, TEXT(F18/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G18, TEXT(F18/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -929,12 +931,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified Narrative Reporting Implementer</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
+          <t>Oracle Narrative Reporting 2026 Implementation Professional (1Z0-1083-26)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -949,7 +951,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="2">
-        <f>IF(G19, TEXT(F19/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G19, TEXT(F19/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -961,27 +963,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Enterprise Data Management Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
+          <t>Integrating Data in Cloud EPM</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>12h 25m</t>
+          <t>4h 43m</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>745</v>
+        <v>283</v>
       </c>
       <c r="G20" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H20" s="2">
-        <f>IF(G20, TEXT(F20/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G20, TEXT(F20/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -993,27 +995,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Enterprise Data Management Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>What's New in Enterprise Data Management</t>
+          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2h 1m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="G21" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H21" s="2">
-        <f>IF(G21, TEXT(F21/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G21, TEXT(F21/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1030,22 +1032,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>12h 25m</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>158</v>
+        <v>745</v>
       </c>
       <c r="G22" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H22" s="2">
-        <f>IF(G22, TEXT(F22/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G22, TEXT(F22/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1062,22 +1064,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Oracle Enterprise Data Management Cloud 2025 Implementation Professional (1Z0-1086-25-JPN)</t>
+          <t>What's New in Enterprise Data Management</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>1h 31m</t>
+          <t>2h 1m</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>91</v>
+        <v>121</v>
       </c>
       <c r="G23" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H23" s="2">
-        <f>IF(G23, TEXT(F23/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G23, TEXT(F23/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1094,22 +1096,22 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Oracle Enterprise Data Management Cloud 2026 Implementation Professional (1Z0-1086-26)</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>90</v>
+        <v>158</v>
       </c>
       <c r="G24" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H24" s="2">
-        <f>IF(G24, TEXT(F24/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G24, TEXT(F24/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1121,27 +1123,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Planning Implementer</t>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM: Planning Implementation</t>
+          <t>Oracle Enterprise Data Management Cloud 2025 Implementation Professional (1Z0-1086-25-JPN)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>10h 17m</t>
+          <t>1h 31m</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>617</v>
+        <v>91</v>
       </c>
       <c r="G25" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H25" s="2">
-        <f>IF(G25, TEXT(F25/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G25, TEXT(F25/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1153,27 +1155,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Become a Certified Planning Implementer</t>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM: Administering Planning Modules</t>
+          <t>Oracle Enterprise Data Management Cloud 2026 Implementation Professional (1Z0-1086-26)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>8h 20m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>500</v>
+        <v>90</v>
       </c>
       <c r="G26" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H26" s="2">
-        <f>IF(G26, TEXT(F26/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G26, TEXT(F26/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1190,22 +1192,22 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Oracle SmartView For Planning</t>
+          <t>Oracle Cloud EPM: Planning Implementation</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2h 40m</t>
+          <t>10h 17m</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>160</v>
+        <v>617</v>
       </c>
       <c r="G27" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H27" s="2">
-        <f>IF(G27, TEXT(F27/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G27, TEXT(F27/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1222,22 +1224,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>What's New in Planning</t>
+          <t>Oracle Cloud EPM: Administering Planning Modules</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>41m</t>
+          <t>8h 20m</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>41</v>
+        <v>500</v>
       </c>
       <c r="G28" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H28" s="2">
-        <f>IF(G28, TEXT(F28/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G28, TEXT(F28/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1254,150 +1256,152 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Oracle SmartView For Planning</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>2h 40m</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G29" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H29" s="2">
-        <f>IF(G29, TEXT(F29/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G29, TEXT(F29/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Pigments Learning</t>
+          <t>Oracle EPM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Pigment Essentials for Business Users</t>
+          <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Pigment Solution Overview</t>
+          <t>What's New in Planning</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>41m</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="G30" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H30" s="2">
-        <f>IF(G30, TEXT(F30/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G30, TEXT(F30/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Pigments Learning</t>
+          <t>Oracle EPM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Pigment Essentials for Business Users</t>
+          <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Pigment Applications</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="G31" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H31" s="2">
-        <f>IF(G31, TEXT(F31/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G31, TEXT(F31/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Business Users</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Pigment Boards</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>2m</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H32" s="2">
-        <f>IF(G32, TEXT(F32/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>Oracle EPM</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr"/>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Planning 2025 Implementation Professional (1Z0-1080-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>1h 31m</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="n">
+        <v>91</v>
+      </c>
+      <c r="G32" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" s="0">
+        <f>IF(G32, TEXT(F32/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Business Users</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Creating Private and Public Comments</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>3m</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H33" s="2">
-        <f>IF(G33, TEXT(F33/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>Oracle EPM</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr"/>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Planning + AI 2026 Implementation Professional (1Z0-1080-26)</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>1h 30m</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="G33" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H33" s="0">
+        <f>IF(G33, TEXT(F33/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1414,22 +1418,22 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Inputting Data</t>
+          <t>Pigment Solution Overview</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>3m</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G34" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H34" s="2">
-        <f>IF(G34, TEXT(F34/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G34, TEXT(F34/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1446,22 +1450,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Board Page Selectors</t>
+          <t>Pigment Applications</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>3m</t>
+          <t>2m</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G35" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H35" s="2">
-        <f>IF(G35, TEXT(F35/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G35, TEXT(F35/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1478,22 +1482,22 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Widget Page Selectors</t>
+          <t>Pigment Boards</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>3m</t>
+          <t>2m</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H36" s="2">
-        <f>IF(G36, TEXT(F36/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G36, TEXT(F36/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1510,22 +1514,22 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Changing a Widget View</t>
+          <t>Creating Private and Public Comments</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>3m</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H37" s="2">
-        <f>IF(G37, TEXT(F37/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G37, TEXT(F37/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1542,22 +1546,22 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Downloading Data From Pigment</t>
+          <t>Inputting Data</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>3m</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="2" t="b">
         <v>1</v>
       </c>
       <c r="H38" s="2">
-        <f>IF(G38, TEXT(F38/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G38, TEXT(F38/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1569,155 +1573,155 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>Pigment Essentials for Business Users</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Board Page Selectors</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>3m</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H39" s="2">
+        <f>IF(G39, TEXT(F39/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Pigment Essentials for Business Users</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Widget Page Selectors</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>3m</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H40" s="2">
+        <f>IF(G40, TEXT(F40/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Pigment Essentials for Business Users</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Changing a Widget View</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" s="2">
+        <f>IF(G41, TEXT(F41/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Pigment Essentials for Business Users</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Downloading Data From Pigment</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" s="2">
+        <f>IF(G42, TEXT(F42/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
           <t>Pigment Essentials for Modelers</t>
         </is>
       </c>
-      <c r="D39" s="0" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>Pigment Solution Overview</t>
         </is>
       </c>
-      <c r="E39" s="0" t="inlineStr">
+      <c r="E43" s="0" t="inlineStr">
         <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="F43" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H39" s="2">
-        <f>IF(G39, TEXT(F39/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B40" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Modelers</t>
-        </is>
-      </c>
-      <c r="D40" s="0" t="inlineStr">
-        <is>
-          <t>Pigment and Multidimensionality</t>
-        </is>
-      </c>
-      <c r="E40" s="0" t="inlineStr">
-        <is>
-          <t>10m</t>
-        </is>
-      </c>
-      <c r="F40" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G40" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H40" s="0">
-        <f>IF(G40, TEXT(F40/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B41" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Modelers</t>
-        </is>
-      </c>
-      <c r="D41" s="0" t="inlineStr">
-        <is>
-          <t>Explore the Workspace</t>
-        </is>
-      </c>
-      <c r="E41" s="0" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="F41" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="G41" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H41" s="0">
-        <f>IF(G41, TEXT(F41/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B42" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Modelers</t>
-        </is>
-      </c>
-      <c r="D42" s="0" t="inlineStr">
-        <is>
-          <t>Build Your First Application</t>
-        </is>
-      </c>
-      <c r="E42" s="0" t="inlineStr">
-        <is>
-          <t>20m</t>
-        </is>
-      </c>
-      <c r="F42" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="G42" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H42" s="0">
-        <f>IF(G42, TEXT(F42/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B43" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Essentials for Modelers</t>
-        </is>
-      </c>
-      <c r="D43" s="0" t="inlineStr">
-        <is>
-          <t>Work with Widgets on Boards</t>
-        </is>
-      </c>
-      <c r="E43" s="0" t="inlineStr">
-        <is>
-          <t>10m</t>
-        </is>
-      </c>
-      <c r="F43" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G43" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H43" s="0">
-        <f>IF(G43, TEXT(F43/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="G43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H43" s="2">
+        <f>IF(G43, TEXT(F43/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1734,22 +1738,22 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>Formula Structure and Syntax</t>
+          <t>Pigment and Multidimensionality</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>10m</t>
         </is>
       </c>
       <c r="F44" s="0" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G44" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="0">
-        <f>IF(G44, TEXT(F44/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G44, TEXT(F44/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1766,22 +1770,22 @@
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>Use Modifiers in Formulas</t>
+          <t>Explore the Workspace</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>7m</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="F45" s="0" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G45" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H45" s="0">
-        <f>IF(G45, TEXT(F45/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G45, TEXT(F45/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1798,22 +1802,22 @@
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>Formula Operations and Aligned Block Dimensions</t>
+          <t>Build Your First Application</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>10m</t>
+          <t>20m</t>
         </is>
       </c>
       <c r="F46" s="0" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G46" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H46" s="0">
-        <f>IF(G46, TEXT(F46/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G46, TEXT(F46/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1830,54 +1834,54 @@
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>Please let us know what you think!</t>
+          <t>Work with Widgets on Boards</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>10m</t>
         </is>
       </c>
       <c r="F47" s="0" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G47" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H47" s="0">
-        <f>IF(G47, TEXT(F47/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G47, TEXT(F47/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>From Process to Experience: UX Design Journey</t>
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Essentials for Modelers</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>Identify Stakeholder Needs for a Board</t>
+          <t>Formula Structure and Syntax</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>20m</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G48" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H48" s="2">
-        <f>IF(G48, TEXT(F48/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="G48" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H48" s="0">
+        <f>IF(G48, TEXT(F48/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1889,27 +1893,27 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>From Process to Experience: UX Design Journey</t>
+          <t>Pigment Essentials for Modelers</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>Work with Widgets on Boards</t>
+          <t>Use Modifiers in Formulas</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>10m</t>
+          <t>7m</t>
         </is>
       </c>
       <c r="F49" s="0" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G49" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H49" s="0">
-        <f>IF(G49, TEXT(F49/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G49, TEXT(F49/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1921,27 +1925,27 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>From Process to Experience: UX Design Journey</t>
+          <t>Pigment Essentials for Modelers</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>When to Use the Different Types of Widgets on Boards</t>
+          <t>Formula Operations and Aligned Block Dimensions</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>30m</t>
+          <t>10m</t>
         </is>
       </c>
       <c r="F50" s="0" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G50" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H50" s="0">
-        <f>IF(G50, TEXT(F50/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G50, TEXT(F50/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -1953,59 +1957,59 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
+          <t>Pigment Essentials for Modelers</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Please let us know what you think!</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H51" s="0">
+        <f>IF(G51, TEXT(F51/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
           <t>From Process to Experience: UX Design Journey</t>
         </is>
       </c>
-      <c r="D51" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Lists</t>
-        </is>
-      </c>
-      <c r="E51" s="0" t="inlineStr">
-        <is>
-          <t>3m</t>
-        </is>
-      </c>
-      <c r="F51" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G51" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H51" s="0">
-        <f>IF(G51, TEXT(F51/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B52" s="0" t="inlineStr">
-        <is>
-          <t>From Process to Experience: UX Design Journey</t>
-        </is>
-      </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>Pigment Lists on Boards</t>
+          <t>Identify Stakeholder Needs for a Board</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>3m</t>
-        </is>
-      </c>
-      <c r="F52" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G52" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H52" s="0">
-        <f>IF(G52, TEXT(F52/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>20m</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H52" s="2">
+        <f>IF(G52, TEXT(F52/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2022,22 +2026,22 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>Pigment Charts</t>
+          <t>Work with Widgets on Boards</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>10m</t>
         </is>
       </c>
       <c r="F53" s="0" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G53" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H53" s="0">
-        <f>IF(G53, TEXT(F53/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G53, TEXT(F53/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2054,22 +2058,22 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>Page Selectors on Boards</t>
+          <t>When to Use the Different Types of Widgets on Boards</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>3m</t>
+          <t>30m</t>
         </is>
       </c>
       <c r="F54" s="0" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G54" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H54" s="0">
-        <f>IF(G54, TEXT(F54/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G54, TEXT(F54/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2086,22 +2090,22 @@
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>Adjusting Page Selectors for Business users</t>
+          <t>Pigment Lists</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>3m</t>
         </is>
       </c>
       <c r="F55" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G55" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H55" s="0">
-        <f>IF(G55, TEXT(F55/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G55, TEXT(F55/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2118,22 +2122,22 @@
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>Pigment Automations</t>
+          <t>Pigment Lists on Boards</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>3m</t>
         </is>
       </c>
       <c r="F56" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G56" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H56" s="0">
-        <f>IF(G56, TEXT(F56/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G56, TEXT(F56/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2150,59 +2154,54 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Build Boards from a Mock-up</t>
+          <t>Pigment Charts</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>45m</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="F57" s="0" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G57" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H57" s="0">
-        <f>IF(G57, TEXT(F57/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G57, TEXT(F57/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
-        </is>
-      </c>
-      <c r="C58" s="0" t="inlineStr">
-        <is>
-          <t>Read and Interpret Formulas</t>
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>From Process to Experience: UX Design Journey</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>Three Essential Elements for Pigment Formulas</t>
+          <t>Page Selectors on Boards</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G58" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H58" s="2">
-        <f>IF(G58, TEXT(F58/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>3m</t>
+        </is>
+      </c>
+      <c r="F58" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G58" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H58" s="0">
+        <f>IF(G58, TEXT(F58/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2214,32 +2213,27 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
-        </is>
-      </c>
-      <c r="C59" s="0" t="inlineStr">
-        <is>
-          <t>Read and Interpret Formulas</t>
+          <t>From Process to Experience: UX Design Journey</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>Anatomy of a Metric</t>
+          <t>Adjusting Page Selectors for Business users</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>3m</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="F59" s="0" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G59" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H59" s="0">
-        <f>IF(G59, TEXT(F59/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G59, TEXT(F59/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2251,32 +2245,27 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
-        </is>
-      </c>
-      <c r="C60" s="0" t="inlineStr">
-        <is>
-          <t>Read and Interpret Formulas</t>
+          <t>From Process to Experience: UX Design Journey</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>Introduction to Pigment Formulas</t>
+          <t>Pigment Automations</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>7m</t>
+          <t>2m</t>
         </is>
       </c>
       <c r="F60" s="0" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G60" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H60" s="0">
-        <f>IF(G60, TEXT(F60/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G60, TEXT(F60/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2288,69 +2277,64 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
+          <t>From Process to Experience: UX Design Journey</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>Build Boards from a Mock-up</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>45m</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="G61" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H61" s="0">
+        <f>IF(G61, TEXT(F61/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
           <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
         </is>
       </c>
-      <c r="C61" s="0" t="inlineStr">
+      <c r="C62" s="0" t="inlineStr">
         <is>
           <t>Read and Interpret Formulas</t>
         </is>
       </c>
-      <c r="D61" s="0" t="inlineStr">
-        <is>
-          <t>Basics of Formula Writing</t>
-        </is>
-      </c>
-      <c r="E61" s="0" t="inlineStr">
-        <is>
-          <t>40m</t>
-        </is>
-      </c>
-      <c r="F61" s="0" t="n">
-        <v>40</v>
-      </c>
-      <c r="G61" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H61" s="0">
-        <f>IF(G61, TEXT(F61/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B62" s="0" t="inlineStr">
-        <is>
-          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
-        </is>
-      </c>
-      <c r="C62" s="0" t="inlineStr">
-        <is>
-          <t>Read and Interpret Formulas</t>
-        </is>
-      </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>Introduction to Modifiers</t>
+          <t>Three Essential Elements for Pigment Formulas</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>11m</t>
-        </is>
-      </c>
-      <c r="F62" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G62" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H62" s="0">
-        <f>IF(G62, TEXT(F62/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G62" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" s="2">
+        <f>IF(G62, TEXT(F62/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2372,22 +2356,22 @@
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>Use Functions in a Formula Activity</t>
+          <t>Anatomy of a Metric</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>45m</t>
+          <t>3m</t>
         </is>
       </c>
       <c r="F63" s="0" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="G63" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H63" s="0">
-        <f>IF(G63, TEXT(F63/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G63, TEXT(F63/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2409,22 +2393,22 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>Formula Playground Activity</t>
+          <t>Introduction to Pigment Formulas</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>40m</t>
+          <t>7m</t>
         </is>
       </c>
       <c r="F64" s="0" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="G64" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H64" s="0">
-        <f>IF(G64, TEXT(F64/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G64, TEXT(F64/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2446,22 +2430,22 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>Formula Wizard Activity</t>
+          <t>Basics of Formula Writing</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>30m</t>
+          <t>40m</t>
         </is>
       </c>
       <c r="F65" s="0" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G65" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H65" s="0">
-        <f>IF(G65, TEXT(F65/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G65, TEXT(F65/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2483,22 +2467,22 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>Read and Interpret Formulas Quiz</t>
+          <t>Introduction to Modifiers</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>20m</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="F66" s="0" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G66" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H66" s="0">
-        <f>IF(G66, TEXT(F66/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G66, TEXT(F66/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2515,27 +2499,27 @@
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>Align Block Dimensions for Formulas</t>
+          <t>Read and Interpret Formulas</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>Formula Operations and Aligned Block Dimensions</t>
+          <t>Use Functions in a Formula Activity</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>10m</t>
+          <t>45m</t>
         </is>
       </c>
       <c r="F67" s="0" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="G67" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H67" s="0">
-        <f>IF(G67, TEXT(F67/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G67, TEXT(F67/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2552,27 +2536,27 @@
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>Align Block Dimensions for Formulas</t>
+          <t>Read and Interpret Formulas</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>Modifiers for Misalignment</t>
+          <t>Formula Playground Activity</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>60m</t>
+          <t>40m</t>
         </is>
       </c>
       <c r="F68" s="0" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G68" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H68" s="0">
-        <f>IF(G68, TEXT(F68/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G68, TEXT(F68/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2589,27 +2573,27 @@
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>Align Block Dimensions for Formulas</t>
+          <t>Read and Interpret Formulas</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>Interactive Source to Target Mapping Tool</t>
+          <t>Formula Wizard Activity</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>30m</t>
         </is>
       </c>
       <c r="F69" s="0" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G69" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H69" s="0">
-        <f>IF(G69, TEXT(F69/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G69, TEXT(F69/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2626,27 +2610,27 @@
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>Align Block Dimensions for Formulas</t>
+          <t>Read and Interpret Formulas</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Work with Dimensionality in Formulas</t>
+          <t>Read and Interpret Formulas Quiz</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>1h 50m</t>
+          <t>20m</t>
         </is>
       </c>
       <c r="F70" s="0" t="n">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="G70" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H70" s="0">
-        <f>IF(G70, TEXT(F70/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G70, TEXT(F70/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2668,22 +2652,22 @@
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>Align Block Dimensions for Formula Operations</t>
+          <t>Formula Operations and Aligned Block Dimensions</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>60m</t>
+          <t>10m</t>
         </is>
       </c>
       <c r="F71" s="0" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="G71" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H71" s="0">
-        <f>IF(G71, TEXT(F71/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G71, TEXT(F71/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2705,22 +2689,22 @@
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>Please let us know what you think!</t>
+          <t>Modifiers for Misalignment</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>2m</t>
+          <t>60m</t>
         </is>
       </c>
       <c r="F72" s="0" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="G72" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H72" s="0">
-        <f>IF(G72, TEXT(F72/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G72, TEXT(F72/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2737,27 +2721,27 @@
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>Write and Test Formulas</t>
+          <t>Align Block Dimensions for Formulas</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>Modifiers for Data Adjustment</t>
+          <t>Interactive Source to Target Mapping Tool</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>60m</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="F73" s="0" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G73" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H73" s="0">
-        <f>IF(G73, TEXT(F73/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G73, TEXT(F73/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2774,27 +2758,27 @@
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>Write and Test Formulas</t>
+          <t>Align Block Dimensions for Formulas</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>ADD, REMOVE and KEEP Modifiers</t>
+          <t>Work with Dimensionality in Formulas</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>60m</t>
+          <t>1h 50m</t>
         </is>
       </c>
       <c r="F74" s="0" t="n">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="G74" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H74" s="0">
-        <f>IF(G74, TEXT(F74/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G74, TEXT(F74/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2811,27 +2795,27 @@
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>Write and Test Formulas</t>
+          <t>Align Block Dimensions for Formulas</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>FILTER &amp; EXCLUDE Modifiers</t>
+          <t>Align Block Dimensions for Formula Operations</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>45m</t>
+          <t>60m</t>
         </is>
       </c>
       <c r="F75" s="0" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="G75" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H75" s="0">
-        <f>IF(G75, TEXT(F75/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G75, TEXT(F75/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2848,27 +2832,27 @@
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>Write and Test Formulas</t>
+          <t>Align Block Dimensions for Formulas</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>BY Modifier</t>
+          <t>Please let us know what you think!</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>2h</t>
+          <t>2m</t>
         </is>
       </c>
       <c r="F76" s="0" t="n">
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="G76" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H76" s="0">
-        <f>IF(G76, TEXT(F76/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G76, TEXT(F76/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2890,22 +2874,22 @@
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>BY -&gt; Modifier</t>
+          <t>Modifiers for Data Adjustment</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>10m</t>
+          <t>60m</t>
         </is>
       </c>
       <c r="F77" s="0" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G77" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H77" s="0">
-        <f>IF(G77, TEXT(F77/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G77, TEXT(F77/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2927,7 +2911,7 @@
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>SELECT Modifier</t>
+          <t>ADD, REMOVE and KEEP Modifiers</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
@@ -2942,7 +2926,7 @@
         <v>1</v>
       </c>
       <c r="H78" s="0">
-        <f>IF(G78, TEXT(F78/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G78, TEXT(F78/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -2964,54 +2948,59 @@
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>Apply Modifiers in Formulas Exercise Guide</t>
+          <t>FILTER &amp; EXCLUDE Modifiers</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>3h 30m</t>
+          <t>45m</t>
         </is>
       </c>
       <c r="F79" s="0" t="n">
-        <v>210</v>
+        <v>45</v>
       </c>
       <c r="G79" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H79" s="0">
-        <f>IF(G79, TEXT(F79/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G79, TEXT(F79/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Pigment Pro Training 2.0</t>
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Basic Path</t>
+          <t>Write and Test Formulas</t>
         </is>
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>Attestation - Pro Training</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G80" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H80" s="2">
-        <f>IF(G80, TEXT(F80/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>BY Modifier</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="F80" s="0" t="n">
+        <v>120</v>
+      </c>
+      <c r="G80" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H80" s="0">
+        <f>IF(G80, TEXT(F80/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3023,27 +3012,32 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training 2.0</t>
+          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Basic Path</t>
+          <t>Write and Test Formulas</t>
         </is>
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>1. Intro &amp; Understanding Business Requirements</t>
+          <t>BY -&gt; Modifier</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>10m</t>
         </is>
       </c>
       <c r="F81" s="0" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G81" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H81" s="0">
-        <f>IF(G81, TEXT(F81/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G81, TEXT(F81/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3055,27 +3049,32 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training 2.0</t>
+          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Basic Path</t>
+          <t>Write and Test Formulas</t>
         </is>
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>2. Data Hub -&gt; Step-by-Step Build</t>
+          <t>SELECT Modifier</t>
+        </is>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
+        <is>
+          <t>60m</t>
         </is>
       </c>
       <c r="F82" s="0" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G82" s="0" t="b">
         <v>1</v>
       </c>
       <c r="H82" s="0">
-        <f>IF(G82, TEXT(F82/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G82, TEXT(F82/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3087,59 +3086,64 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
+          <t>Formula Writing: Unlocking Dimensionality and Calculations</t>
+        </is>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t>Write and Test Formulas</t>
+        </is>
+      </c>
+      <c r="D83" s="0" t="inlineStr">
+        <is>
+          <t>Apply Modifiers in Formulas Exercise Guide</t>
+        </is>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t>3h 30m</t>
+        </is>
+      </c>
+      <c r="F83" s="0" t="n">
+        <v>210</v>
+      </c>
+      <c r="G83" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H83" s="0">
+        <f>IF(G83, TEXT(F83/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
           <t>Pigment Pro Training 2.0</t>
         </is>
       </c>
-      <c r="C83" s="0" t="inlineStr">
+      <c r="C84" s="0" t="inlineStr">
         <is>
           <t>Pigment Pro Training - Basic Path</t>
         </is>
       </c>
-      <c r="D83" s="0" t="inlineStr">
-        <is>
-          <t>3. Workforce Planning</t>
-        </is>
-      </c>
-      <c r="F83" s="0" t="n">
+      <c r="D84" s="0" t="inlineStr">
+        <is>
+          <t>Attestation - Pro Training</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G83" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H83" s="0">
-        <f>IF(G83, TEXT(F83/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="0" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B84" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Pro Training 2.0</t>
-        </is>
-      </c>
-      <c r="C84" s="0" t="inlineStr">
-        <is>
-          <t>Pigment Pro Training - Basic Path</t>
-        </is>
-      </c>
-      <c r="D84" s="0" t="inlineStr">
-        <is>
-          <t>Data Hub &amp; Workforce Planning Assessment</t>
-        </is>
-      </c>
-      <c r="F84" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G84" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="H84" s="0">
-        <f>IF(G84, TEXT(F84/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+      <c r="G84" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H84" s="2">
+        <f>IF(G84, TEXT(F84/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3156,12 +3160,12 @@
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Advanced Path</t>
+          <t>Pigment Pro Training - Basic Path</t>
         </is>
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>4. Connecting the OpEx App</t>
+          <t>1. Intro &amp; Understanding Business Requirements</t>
         </is>
       </c>
       <c r="F85" s="0" t="n">
@@ -3171,7 +3175,7 @@
         <v>1</v>
       </c>
       <c r="H85" s="0">
-        <f>IF(G85, TEXT(F85/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G85, TEXT(F85/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3188,12 +3192,12 @@
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Advanced Path</t>
+          <t>Pigment Pro Training - Basic Path</t>
         </is>
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>Quiz: OpEX Planning</t>
+          <t>2. Data Hub -&gt; Step-by-Step Build</t>
         </is>
       </c>
       <c r="F86" s="0" t="n">
@@ -3203,7 +3207,7 @@
         <v>1</v>
       </c>
       <c r="H86" s="0">
-        <f>IF(G86, TEXT(F86/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G86, TEXT(F86/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3220,12 +3224,12 @@
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Advanced Path</t>
+          <t>Pigment Pro Training - Basic Path</t>
         </is>
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>5. Core Reporting</t>
+          <t>3. Workforce Planning</t>
         </is>
       </c>
       <c r="F87" s="0" t="n">
@@ -3235,7 +3239,7 @@
         <v>1</v>
       </c>
       <c r="H87" s="0">
-        <f>IF(G87, TEXT(F87/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G87, TEXT(F87/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3252,12 +3256,12 @@
       </c>
       <c r="C88" s="0" t="inlineStr">
         <is>
-          <t>Pigment Pro Training - Advanced Path</t>
+          <t>Pigment Pro Training - Basic Path</t>
         </is>
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>Quiz: Core Reporting</t>
+          <t>Data Hub &amp; Workforce Planning Assessment</t>
         </is>
       </c>
       <c r="F88" s="0" t="n">
@@ -3267,7 +3271,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="0">
-        <f>IF(G88, TEXT(F88/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G88, TEXT(F88/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3289,7 +3293,7 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>6. Centralized Security Hub</t>
+          <t>4. Connecting the OpEx App</t>
         </is>
       </c>
       <c r="F89" s="0" t="n">
@@ -3299,7 +3303,7 @@
         <v>1</v>
       </c>
       <c r="H89" s="0">
-        <f>IF(G89, TEXT(F89/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G89, TEXT(F89/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3321,7 +3325,7 @@
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>7. Topline Planning</t>
+          <t>Quiz: OpEX Planning</t>
         </is>
       </c>
       <c r="F90" s="0" t="n">
@@ -3331,7 +3335,7 @@
         <v>1</v>
       </c>
       <c r="H90" s="0">
-        <f>IF(G90, TEXT(F90/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G90, TEXT(F90/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3353,7 +3357,7 @@
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>Quiz: Topline Planning</t>
+          <t>5. Core Reporting</t>
         </is>
       </c>
       <c r="F91" s="0" t="n">
@@ -3363,7 +3367,7 @@
         <v>1</v>
       </c>
       <c r="H91" s="0">
-        <f>IF(G91, TEXT(F91/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G91, TEXT(F91/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3385,7 +3389,7 @@
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>8. Change Requests</t>
+          <t>Quiz: Core Reporting</t>
         </is>
       </c>
       <c r="F92" s="0" t="n">
@@ -3395,7 +3399,7 @@
         <v>1</v>
       </c>
       <c r="H92" s="0">
-        <f>IF(G92, TEXT(F92/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G92, TEXT(F92/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3417,7 +3421,7 @@
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>Final Assessment</t>
+          <t>6. Centralized Security Hub</t>
         </is>
       </c>
       <c r="F93" s="0" t="n">
@@ -3427,39 +3431,39 @@
         <v>1</v>
       </c>
       <c r="H93" s="0">
-        <f>IF(G93, TEXT(F93/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G93, TEXT(F93/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>Pigments Learning</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>Partner Application Builder Certification</t>
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training 2.0</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training - Advanced Path</t>
         </is>
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>In-Person Partner App Builder Workshop</t>
-        </is>
-      </c>
-      <c r="E94" s="0" t="inlineStr">
-        <is>
-          <t>2.5 days</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G94" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H94" s="2">
-        <f>IF(G94, TEXT(F94/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+          <t>7. Topline Planning</t>
+        </is>
+      </c>
+      <c r="F94" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H94" s="0">
+        <f>IF(G94, TEXT(F94/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3471,12 +3475,17 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>Partner Application Builder Certification</t>
+          <t>Pigment Pro Training 2.0</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training - Advanced Path</t>
         </is>
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t>Pigment Partner App Builder Certification &amp; Evaluation</t>
+          <t>Quiz: Topline Planning</t>
         </is>
       </c>
       <c r="F95" s="0" t="n">
@@ -3486,7 +3495,130 @@
         <v>1</v>
       </c>
       <c r="H95" s="0">
-        <f>IF(G95, TEXT(F95/SUMIF($G$2:$G$95, TRUE, $F$2:$F$95), "0.00%"), "0.00%")</f>
+        <f>IF(G95, TEXT(F95/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training 2.0</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training - Advanced Path</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>8. Change Requests</t>
+        </is>
+      </c>
+      <c r="F96" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H96" s="0">
+        <f>IF(G96, TEXT(F96/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training 2.0</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Pro Training - Advanced Path</t>
+        </is>
+      </c>
+      <c r="D97" s="0" t="inlineStr">
+        <is>
+          <t>Final Assessment</t>
+        </is>
+      </c>
+      <c r="F97" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H97" s="0">
+        <f>IF(G97, TEXT(F97/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Partner Application Builder Certification</t>
+        </is>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t>In-Person Partner App Builder Workshop</t>
+        </is>
+      </c>
+      <c r="E98" s="0" t="inlineStr">
+        <is>
+          <t>2.5 days</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G98" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H98" s="2">
+        <f>IF(G98, TEXT(F98/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t>Pigments Learning</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t>Partner Application Builder Certification</t>
+        </is>
+      </c>
+      <c r="D99" s="0" t="inlineStr">
+        <is>
+          <t>Pigment Partner App Builder Certification &amp; Evaluation</t>
+        </is>
+      </c>
+      <c r="F99" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H99" s="0">
+        <f>IF(G99, TEXT(F99/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
@@ -3501,7 +3633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3525,9 +3657,19 @@
           <t>Role</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>PasswordHash</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>MustChangePassword</t>
         </is>
       </c>
     </row>
@@ -3552,10 +3694,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>Lam.Le@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>130685944460738e22df8aee02a0da19$0bd762e5869440d84fb05740ee065eb2e8a11613fb6ca99774680e77106cc01f</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3579,10 +3729,18 @@
           <t>Super User</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>khuong.ngo@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>86df1b9ad52e7f42ffc81fac94b00df0$ce32ec48abd6cac2091d359100e9e6d41d5483e8f5f7152cb0473f8c36f9afae</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3606,10 +3764,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>Wynn.Nguyen@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -3633,10 +3799,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>Wendy.Nguyen@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -3660,10 +3834,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>Hannah.Dinh@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3687,10 +3869,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>Austin.Nguyen@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -3714,10 +3904,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>Mia.Tran@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3741,10 +3939,18 @@
           <t>Employee</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>Trung.Nguyen@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3768,10 +3974,18 @@
           <t>Manager</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>Hanoi.Office@AreteEPM.com</t>
         </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add show password toggle, remove admin footer hint, and reset all passwords to EPM@2026
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3701,7 +3701,7 @@
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>130685944460738e22df8aee02a0da19$0bd762e5869440d84fb05740ee065eb2e8a11613fb6ca99774680e77106cc01f</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G2" s="0" t="b">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>86df1b9ad52e7f42ffc81fac94b00df0$ce32ec48abd6cac2091d359100e9e6d41d5483e8f5f7152cb0473f8c36f9afae</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G3" s="0" t="b">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G4" s="0" t="b">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G5" s="0" t="b">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G6" s="0" t="b">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G7" s="0" t="b">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G8" s="0" t="b">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G9" s="0" t="b">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>c7888617e457914e9a1a25b6c27129e2$0694a1c2b3c8f7245586705d5aa134dcfe3eb863f505328e3dae310019eb7604</t>
+          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
       <c r="G10" s="0" t="b">

</xml_diff>

<commit_message>
feat: Add profile management modal, avatar file upload/URL support, show password toggle for all fields, and forgot-to-login action
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3736,11 +3736,11 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
+          <t>b820fffce7346444a196b3caf30f303d$a96bad452fd9deecb6a587078b6d73982e02380015642b3d70c0f4d46925a118</t>
         </is>
       </c>
       <c r="G3" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
feat: Add user avatar file upload/URL management, show password toggles on all password fields, and forgot-to-login modal flow
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3633,7 +3633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3670,6 +3670,11 @@
       <c r="G1" s="0" t="inlineStr">
         <is>
           <t>MustChangePassword</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>AvatarUrl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Remember Me credentials saving and Manager View-As progress inspection mode without losing session
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3672,7 +3672,7 @@
           <t>MustChangePassword</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="0" t="inlineStr">
         <is>
           <t>AvatarUrl</t>
         </is>
@@ -3746,6 +3746,11 @@
       </c>
       <c r="G3" s="0" t="b">
         <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>/uploads/avatars/11_shared_image.jpg</t>
+        </is>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
feat: Add Edit Enrollment functionality and update workweek summary calculation display
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3747,7 +3747,7 @@
       <c r="G3" s="0" t="b">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t>/uploads/avatars/11_shared_image.jpg</t>
         </is>
@@ -4075,7 +4075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4086,22 +4086,37 @@
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
-          <t>Course Name</t>
+          <t>Target Type</t>
         </is>
       </c>
       <c r="C1" s="0" t="inlineStr">
         <is>
+          <t>Target Name</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="D1" s="0" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Planned End Date</t>
         </is>
       </c>
-      <c r="E1" s="0" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
         <is>
           <t>Workweek Type</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>Daily Hours</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add move module, add module, and delete module features in course management
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3210,21 +3210,21 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Become a Certified Narrative Reporting Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Creating Reports in Cloud EPM</t>
+          <t>Integrating Data in Cloud EPM</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2h 21m</t>
+          <t>4h 43m</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>141</v>
+        <v>283</v>
       </c>
       <c r="G87" t="b">
         <v>1</v>
@@ -3242,21 +3242,21 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Become a Certified Narrative Reporting Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Narrative Reporting Overview and Administration</t>
+          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>1h 39m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G88" t="b">
         <v>1</v>
@@ -3279,19 +3279,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Create and Manage Report Packages in Narrative Reporting</t>
+          <t>Creating Reports in Cloud EPM</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2h 0m</t>
+          <t>2h 21m</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="G89" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H89">
         <f>IF(G89, TEXT(F89/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3311,19 +3311,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>What's New in Narrative Reporting</t>
+          <t>Narrative Reporting Overview and Administration</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>35m</t>
+          <t>1h 39m</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="G90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90">
         <f>IF(G90, TEXT(F90/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3343,19 +3343,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Create and Manage Report Packages in Narrative Reporting</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>2h 0m</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="G91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H91">
         <f>IF(G91, TEXT(F91/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3375,19 +3375,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Oracle Narrative Reporting 2025 Implementation Professional (1Z0-1083-25-JPN)</t>
+          <t>What's New in Narrative Reporting</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>1h 31m</t>
+          <t>35m</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="G92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H92">
         <f>IF(G92, TEXT(F92/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3407,19 +3407,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Oracle Narrative Reporting 2026 Implementation Professional (1Z0-1083-26)</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>90</v>
+        <v>158</v>
       </c>
       <c r="G93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H93">
         <f>IF(G93, TEXT(F93/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3434,24 +3434,24 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Become a Certified PCM Implementer</t>
+          <t>Become a Certified Narrative Reporting Implementer</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM: Enterprise Profitability and Cost Management</t>
+          <t>Oracle Narrative Reporting 2025 Implementation Professional (1Z0-1083-25-JPN)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>14h 20m</t>
+          <t>1h 31m</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>860</v>
+        <v>91</v>
       </c>
       <c r="G94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H94">
         <f>IF(G94, TEXT(F94/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3466,24 +3466,24 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Become a Certified PCM Implementer</t>
+          <t>Become a Certified Narrative Reporting Implementer</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>What's New in Enterprise Profitability and Cost Management</t>
+          <t>Oracle Narrative Reporting 2026 Implementation Professional (1Z0-1083-26)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>47m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="G95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H95">
         <f>IF(G95, TEXT(F95/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3503,19 +3503,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Oracle Cloud EPM: Enterprise Profitability and Cost Management</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>14h 20m</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>158</v>
+        <v>860</v>
       </c>
       <c r="G96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H96">
         <f>IF(G96, TEXT(F96/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3535,19 +3535,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Oracle Profitability and Cost Management 2026 Implementation Professional (1Z0-1082-26)</t>
+          <t>What's New in Enterprise Profitability and Cost Management</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>47m</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="G97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H97">
         <f>IF(G97, TEXT(F97/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3562,24 +3562,24 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified PCM Implementer</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Integrating Data in Cloud EPM</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>4h 43m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="G98" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H98">
         <f>IF(G98, TEXT(F98/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3594,12 +3594,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified PCM Implementer</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
+          <t>Oracle Profitability and Cost Management 2026 Implementation Professional (1Z0-1082-26)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -3611,7 +3611,7 @@
         <v>90</v>
       </c>
       <c r="G99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H99">
         <f>IF(G99, TEXT(F99/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>

</xml_diff>

<commit_message>
Bản có tiếng Việt, đã thêm user và custome course
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -2986,21 +2986,21 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Become a Certified FCC Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Financial Consolidation and Close (FCC): Implementation</t>
+          <t>Integrating Data in Cloud EPM</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>10h 32m</t>
+          <t>4h 43m</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>632</v>
+        <v>283</v>
       </c>
       <c r="G80" t="b">
         <v>1</v>
@@ -3018,21 +3018,21 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Become a Certified FCC Implementer</t>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
+          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>10h 41m</t>
+          <t>1h 30m</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>641</v>
+        <v>90</v>
       </c>
       <c r="G81" t="b">
         <v>1</v>
@@ -3055,16 +3055,16 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Oracle SmartView For Financial Consolidation and Close</t>
+          <t>Financial Consolidation and Close (FCC): Implementation</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2h 40m</t>
+          <t>10h 32m</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>160</v>
+        <v>632</v>
       </c>
       <c r="G82" t="b">
         <v>1</v>
@@ -3087,16 +3087,16 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>What's New in Financial Consolidation and Close</t>
+          <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>25m</t>
+          <t>10h 41m</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>25</v>
+        <v>641</v>
       </c>
       <c r="G83" t="b">
         <v>1</v>
@@ -3119,19 +3119,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>What's New for Common Cloud EPM components</t>
+          <t>Oracle SmartView For Financial Consolidation and Close</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2h 38m</t>
+          <t>2h 40m</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H84">
         <f>IF(G84, TEXT(F84/SUMIF($G$2:$G$99, TRUE, $F$2:$F$99), "0.00%"), "0.00%")</f>
@@ -3151,16 +3151,16 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
+          <t>What's New in Financial Consolidation and Close</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>1h 31m</t>
+          <t>25m</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="G85" t="b">
         <v>1</v>
@@ -3183,16 +3183,16 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
+          <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>1h 30m</t>
+          <t>2h 38m</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>90</v>
+        <v>158</v>
       </c>
       <c r="G86" t="b">
         <v>1</v>
@@ -3210,21 +3210,21 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Integrating Data in Cloud EPM</t>
+          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>4h 43m</t>
+          <t>1h 31m</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>283</v>
+        <v>91</v>
       </c>
       <c r="G87" t="b">
         <v>1</v>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+          <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
+          <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">

</xml_diff>

<commit_message>
feat: 100% translation coverage for all KPI cards, tables, headers, and badges
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -3729,199 +3729,199 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr">
+      <c r="C103" s="0" t="inlineStr"/>
+      <c r="D103" s="0" t="inlineStr">
         <is>
           <t>Financial Consolidation and Close (FCC): Implementation</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E103" s="0" t="inlineStr">
         <is>
           <t>10h 32m</t>
         </is>
       </c>
-      <c r="F103" t="n">
+      <c r="F103" s="0" t="n">
         <v>632</v>
       </c>
-      <c r="G103" t="b">
-        <v>1</v>
-      </c>
-      <c r="H103">
+      <c r="G103" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H103" s="0">
         <f>IF(G103, TEXT(F103/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B104" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr">
+      <c r="C104" s="0" t="inlineStr"/>
+      <c r="D104" s="0" t="inlineStr">
         <is>
           <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E104" s="0" t="inlineStr">
         <is>
           <t>10h 41m</t>
         </is>
       </c>
-      <c r="F104" t="n">
+      <c r="F104" s="0" t="n">
         <v>641</v>
       </c>
-      <c r="G104" t="b">
-        <v>1</v>
-      </c>
-      <c r="H104">
+      <c r="G104" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H104" s="0">
         <f>IF(G104, TEXT(F104/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr">
+      <c r="C105" s="0" t="inlineStr"/>
+      <c r="D105" s="0" t="inlineStr">
         <is>
           <t>What's New in Financial Consolidation and Close</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E105" s="0" t="inlineStr">
         <is>
           <t>25m</t>
         </is>
       </c>
-      <c r="F105" t="n">
+      <c r="F105" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="G105" t="b">
-        <v>1</v>
-      </c>
-      <c r="H105">
+      <c r="G105" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H105" s="0">
         <f>IF(G105, TEXT(F105/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
+      <c r="A106" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B106" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr">
+      <c r="C106" s="0" t="inlineStr"/>
+      <c r="D106" s="0" t="inlineStr">
         <is>
           <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E106" s="0" t="inlineStr">
         <is>
           <t>2h 38m</t>
         </is>
       </c>
-      <c r="F106" t="n">
+      <c r="F106" s="0" t="n">
         <v>158</v>
       </c>
-      <c r="G106" t="b">
-        <v>1</v>
-      </c>
-      <c r="H106">
+      <c r="G106" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H106" s="0">
         <f>IF(G106, TEXT(F106/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
+      <c r="A107" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B107" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr">
+      <c r="C107" s="0" t="inlineStr"/>
+      <c r="D107" s="0" t="inlineStr">
         <is>
           <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E107" s="0" t="inlineStr">
         <is>
           <t>1h 31m</t>
         </is>
       </c>
-      <c r="F107" t="n">
+      <c r="F107" s="0" t="n">
         <v>91</v>
       </c>
-      <c r="G107" t="b">
-        <v>1</v>
-      </c>
-      <c r="H107">
+      <c r="G107" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H107" s="0">
         <f>IF(G107, TEXT(F107/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
+      <c r="A108" s="0" t="inlineStr">
         <is>
           <t>Oracle EPM - Q3 2026 - Fast learning</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B108" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr">
+      <c r="C108" s="0" t="inlineStr"/>
+      <c r="D108" s="0" t="inlineStr">
         <is>
           <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E108" s="0" t="inlineStr">
         <is>
           <t>1h 30m</t>
         </is>
       </c>
-      <c r="F108" t="n">
+      <c r="F108" s="0" t="n">
         <v>90</v>
       </c>
-      <c r="G108" t="b">
-        <v>1</v>
-      </c>
-      <c r="H108">
+      <c r="G108" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H108" s="0">
         <f>IF(G108, TEXT(F108/SUMIF($G$2:$G$119, TRUE, $F$2:$F$119), "0.00%"), "0.00%")</f>
         <v/>
       </c>
@@ -4665,7 +4665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4717,6 +4717,1366 @@
       <c r="J1" s="0" t="inlineStr">
         <is>
           <t>Tracking Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr"/>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="J2" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr"/>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>What's New in Enterprise Data Management</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr"/>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J4" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr"/>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Enterprise Data Management Cloud 2025 Implementation Professional (1Z0-1086-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J5" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr"/>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Enterprise Data Management Cloud 2026 Implementation Professional (1Z0-1086-26)</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J6" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr"/>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM: Planning Implementation</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>46254</v>
+      </c>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr"/>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM: Administering Planning Modules</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>46256</v>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr"/>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Oracle SmartView For Planning</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>46256</v>
+      </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr"/>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>What's New in Planning</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr"/>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J11" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr"/>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Planning 2025 Implementation Professional (1Z0-1080-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr"/>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Planning + AI 2026 Implementation Professional (1Z0-1080-26)</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr"/>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Integrating Data in Cloud EPM</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>46260</v>
+      </c>
+      <c r="J14" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr"/>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>46260</v>
+      </c>
+      <c r="J15" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr"/>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Financial Consolidation and Close (FCC): Implementation</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>46262</v>
+      </c>
+      <c r="J16" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr"/>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="J17" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr"/>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>What's New in Financial Consolidation and Close</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="J18" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr"/>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J19" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr"/>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J20" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr"/>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J21" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>What's New in Enterprise Data Management</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>46249</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Oracle Enterprise Data Management Cloud 2025 Implementation Professional (1Z0-1086-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Oracle Enterprise Data Management Cloud 2026 Implementation Professional (1Z0-1086-26)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>46251</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM: Planning Implementation</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>46254</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM: Administering Planning Modules</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>46256</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Oracle SmartView For Planning</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>46256</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>What's New in Planning</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Oracle Planning 2025 Implementation Professional (1Z0-1080-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>46258</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Become a Certified Planning Implementer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Oracle Planning + AI 2026 Implementation Professional (1Z0-1080-26)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Integrating Data in Cloud EPM</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>46260</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>46260</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Financial Consolidation and Close (FCC): Implementation</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>46262</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>What's New in Financial Consolidation and Close</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>46266</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>What's New for Common Cloud EPM components</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Become a Certified FCC Implementer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>On-track</t>
         </is>
       </c>
     </row>
@@ -4731,7 +6091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4776,6 +6136,70 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Oracle EPM - Q3 2026 - Fast learning</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Oracle EPM - Q3 2026 - Fast learning</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>46267</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Map all i18n translation keys properly to eliminate raw code key display
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -4392,7 +4392,7 @@
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>khuong.ngo@AreteEPM.com</t>
+          <t>Khuong.Ngo@AreteEPM.com</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
@@ -5401,680 +5401,680 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr"/>
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="4" t="n">
         <v>46249</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr"/>
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>What's New in Enterprise Data Management</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="4" t="n">
         <v>46249</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr"/>
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr"/>
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Oracle Enterprise Data Management Cloud 2025 Implementation Professional (1Z0-1086-25-JPN)</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Enterprise Data Management Implementer</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr"/>
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Oracle Enterprise Data Management Cloud 2026 Implementation Professional (1Z0-1086-26)</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>46251</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr"/>
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Oracle Cloud EPM: Planning Implementation</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="4" t="n">
         <v>46254</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr"/>
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Oracle Cloud EPM: Administering Planning Modules</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="4" t="n">
         <v>46256</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr"/>
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Oracle SmartView For Planning</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="4" t="n">
         <v>46256</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr"/>
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>What's New in Planning</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="4" t="n">
         <v>46258</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr"/>
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>46258</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr"/>
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Oracle Planning 2025 Implementation Professional (1Z0-1080-25-JPN)</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F32" t="n">
+      <c r="F32" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="4" t="n">
         <v>46258</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Planning Implementer</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr"/>
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>Oracle Planning + AI 2026 Implementation Professional (1Z0-1080-26)</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="4" t="n">
         <v>46259</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr"/>
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Integrating Data in Cloud EPM</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I34" s="4" t="n">
         <v>46260</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>Become a Certified Oracle Cloud EPM Data Integration Implementer</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr"/>
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>Oracle Cloud EPM Data Integration 2026 Implementation Professional (1Z0-1133-26)</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="4" t="n">
         <v>46260</v>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr"/>
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Financial Consolidation and Close (FCC): Implementation</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F36" t="n">
+      <c r="F36" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="4" t="n">
         <v>46262</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr"/>
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Financial Consolidation and Close (FCC): Designing the Close Process</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="F37" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr"/>
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>What's New in Financial Consolidation and Close</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F38" t="n">
+      <c r="F38" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr"/>
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>What's New for Common Cloud EPM components</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>46267</v>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr"/>
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>Oracle Financial Consolidation and Close 2025 Implementation Professional (1Z0-1081-25-JPN)</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
         <v>46267</v>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>Become a Certified FCC Implementer</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr"/>
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>Oracle Financial Consolidation and Close 2026 Implementation Professional (1Z0-1081-26)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="0" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="4" t="n">
         <v>46267</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>

</xml_diff>

<commit_message>
feat: Add full English translation to progress modal and implement smart status date/percent automation
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -4665,7 +4665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6075,6 +6075,46 @@
         <v>46267</v>
       </c>
       <c r="J41" s="0" t="inlineStr">
+        <is>
+          <t>On-track</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>Become a Certified Enterprise Data Management Implementer</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr"/>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Manage &amp; Govern Enterprise Data Assets with Enterprise Data Management Cloud</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>46246</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>46247</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>46247</v>
+      </c>
+      <c r="J42" s="0" t="inlineStr">
         <is>
           <t>On-track</t>
         </is>

</xml_diff>

<commit_message>
fix: Link Plan enrollment to course modules in profile view and pass target username to progress modal
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -4746,7 +4746,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>46249</v>
+        <v>46246</v>
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
@@ -4780,7 +4780,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>46249</v>
+        <v>46246</v>
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
@@ -4814,7 +4814,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>46251</v>
+        <v>46247</v>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
@@ -4916,7 +4916,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>46254</v>
+        <v>46251</v>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
@@ -4950,7 +4950,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>46256</v>
+        <v>46253</v>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>46256</v>
+        <v>46253</v>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
@@ -5018,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>46258</v>
+        <v>46254</v>
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
@@ -5052,7 +5052,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>46258</v>
+        <v>46254</v>
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>46258</v>
+        <v>46254</v>
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>46259</v>
+        <v>46255</v>
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
@@ -5222,7 +5222,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>46262</v>
+        <v>46259</v>
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
@@ -5290,7 +5290,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
@@ -5324,7 +5324,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
@@ -5358,7 +5358,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
@@ -5392,7 +5392,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
@@ -6193,10 +6193,10 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>46246</v>
+        <v>46242</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>46267</v>
+        <v>46263</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
fix: Correct tracking speed evaluation logic for Not Started modules reaching or exceeding planned target date
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -4746,11 +4746,11 @@
         <v>0</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>On-track</t>
+          <t>Slow</t>
         </is>
       </c>
     </row>
@@ -4780,11 +4780,11 @@
         <v>0</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t>On-track</t>
+          <t>Slow</t>
         </is>
       </c>
     </row>
@@ -4814,11 +4814,11 @@
         <v>0</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t>On-track</t>
+          <t>Slow</t>
         </is>
       </c>
     </row>
@@ -4848,11 +4848,11 @@
         <v>0</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>On-track</t>
+          <t>Slow</t>
         </is>
       </c>
     </row>
@@ -4882,11 +4882,11 @@
         <v>0</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t>On-track</t>
+          <t>Slow</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
@@ -4950,7 +4950,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
@@ -5018,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
@@ -5052,7 +5052,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
@@ -5120,7 +5120,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
@@ -5222,7 +5222,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
@@ -5290,7 +5290,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
@@ -5324,7 +5324,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
@@ -5358,7 +5358,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
@@ -5392,7 +5392,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
@@ -6193,10 +6193,10 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>46242</v>
+        <v>46240</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
fix: Remove blocking browser alert popup and set MustChangePassword=0 to enable smooth modal clicks
</commit_message>
<xml_diff>
--- a/sheet.xlsx
+++ b/sheet.xlsx
@@ -4365,8 +4365,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G2" s="0" t="b">
-        <v>1</v>
+      <c r="G2" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -4400,7 +4400,7 @@
           <t>b820fffce7346444a196b3caf30f303d$a96bad452fd9deecb6a587078b6d73982e02380015642b3d70c0f4d46925a118</t>
         </is>
       </c>
-      <c r="G3" s="0" t="b">
+      <c r="G3" s="0" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -4440,8 +4440,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G4" s="0" t="b">
-        <v>1</v>
+      <c r="G4" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4475,8 +4475,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G5" s="0" t="b">
-        <v>1</v>
+      <c r="G5" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4510,8 +4510,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G6" s="0" t="b">
-        <v>1</v>
+      <c r="G6" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -4545,8 +4545,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G7" s="0" t="b">
-        <v>1</v>
+      <c r="G7" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4580,8 +4580,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G8" s="0" t="b">
-        <v>1</v>
+      <c r="G8" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4615,8 +4615,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G9" s="0" t="b">
-        <v>1</v>
+      <c r="G9" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4650,8 +4650,8 @@
           <t>7239983ad4895a30fc6ff854fe757073$7b71a2f00ab59d08b52e20f66c68b0b53a301dd33314eb42625d8b722c82a76b</t>
         </is>
       </c>
-      <c r="G10" s="0" t="b">
-        <v>1</v>
+      <c r="G10" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4739,11 +4739,14 @@
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F2" s="0" t="n">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>46246</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>46244</v>

</xml_diff>